<commit_message>
Add Lenovo BRDA DCG (XLSX) parser
Reads the legacy .xls (OLE Compound Document) via ExcelDataReader,
extracts parent CTO items with their child components, and routes
output through AnzGenericWriter for the No Calculation / Uplift
templates (selectable per parse, same as HP).

- New parser LenovoBrdaDcgXlsxParser: anchor-based header (PN /
  Description / Requested Quantity), Total: footer terminator,
  PARENT classified by unit price > 0 (an explicit 0.0 cell stays a
  CHILD, e.g. 5374CM1 Configuration Instruction rows).
- LineSequence: integer for parents (1, 2, ...), parent.NN for
  children (1.01, 1.02, ...).
- ParseService accepts .xls extension and OLE magic bytes
  (D0 CF 11 E0 A1 B1 1A E1); HistoryEndpoints maps .xls MIME.
- Sample BRDAD010458440.xls + goldens for both CRM templates;
  parser + writer tests; spec at docs/lenovo_brda_dcg_xlsx.md.
- Test suite: 157 passing (90 parsing + 67 API).
</commit_message>
<xml_diff>
--- a/samples/outputs/BRDAS010260417V1_parsed.xlsx
+++ b/samples/outputs/BRDAS010260417V1_parsed.xlsx
@@ -123,504 +123,501 @@
     <x:t>2.01</x:t>
   </x:si>
   <x:si>
+    <x:t>C1XE</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 1U V4 10x2.5" Chassis</x:t>
+  </x:si>
+  <x:si>
     <x:t>2.02</x:t>
   </x:si>
   <x:si>
-    <x:t>C1XE</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 1U V4 10x2.5" Chassis</x:t>
+    <x:t>C3JB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem General Computing Power Efficiency -</x:t>
   </x:si>
   <x:si>
     <x:t>2.03</x:t>
   </x:si>
   <x:si>
-    <x:t>C3JB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem General Computing Power Efficiency -</x:t>
+    <x:t>BVGL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Data Center Environment 30 Degree Celsius / 86 Degree Fahrenheit</x:t>
   </x:si>
   <x:si>
     <x:t>2.04</x:t>
   </x:si>
   <x:si>
-    <x:t>BVGL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Data Center Environment 30 Degree Celsius / 86 Degree Fahrenheit</x:t>
+    <x:t>C659</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Intel Xeon 6527P 24C 255W 3.0GHz Processor</x:t>
   </x:si>
   <x:si>
     <x:t>2.05</x:t>
   </x:si>
   <x:si>
-    <x:t>C659</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Intel Xeon 6527P 24C 255W 3.0GHz Processor</x:t>
+    <x:t>C1XJ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 1U V4 Performance Heatsink</x:t>
   </x:si>
   <x:si>
     <x:t>2.06</x:t>
   </x:si>
   <x:si>
-    <x:t>C1XJ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 1U V4 Performance Heatsink</x:t>
+    <x:t>C0TQ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 64GB TruDDR5 6400MHz (2Rx4) RDIMM</x:t>
   </x:si>
   <x:si>
     <x:t>2.07</x:t>
   </x:si>
   <x:si>
-    <x:t>C0TQ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 64GB TruDDR5 6400MHz (2Rx4) RDIMM</x:t>
+    <x:t>5977</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Select Storage devices configured RAID required no -</x:t>
   </x:si>
   <x:si>
     <x:t>2.08</x:t>
   </x:si>
   <x:si>
-    <x:t>5977</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Select Storage devices configured RAID required no -</x:t>
+    <x:t>CCCZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem M.2 RAID B550p-2HS SATA/NVMe Enablement Kit</x:t>
   </x:si>
   <x:si>
     <x:t>2.09</x:t>
   </x:si>
   <x:si>
-    <x:t>CCCZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem M.2 RAID B550p-2HS SATA/NVMe Enablement Kit</x:t>
+    <x:t>C286</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem M.2 VA 480GB Read Intensive NVMe NHS SSD</x:t>
   </x:si>
   <x:si>
     <x:t>2.10</x:t>
   </x:si>
   <x:si>
-    <x:t>C286</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem M.2 VA 480GB Read Intensive NVMe NHS SSD</x:t>
+    <x:t>BCD4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem Intel E810-DA2 10/25GbE SFP28 2-Port OCP Ethernet Adapter</x:t>
   </x:si>
   <x:si>
     <x:t>2.11</x:t>
   </x:si>
   <x:si>
-    <x:t>BCD4</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem Intel E810-DA2 10/25GbE SFP28 2-Port OCP Ethernet Adapter</x:t>
+    <x:t>BCD6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem Intel E810-DA2 10/25GbE SFP28 2-Port PCIe Ethernet Adapter</x:t>
   </x:si>
   <x:si>
     <x:t>2.12</x:t>
   </x:si>
   <x:si>
-    <x:t>BCD6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem Intel E810-DA2 10/25GbE SFP28 2-Port PCIe Ethernet Adapter</x:t>
+    <x:t>BYBJ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem Finisar Dual Rate 10G/25G SR SFP28 Transceiver</x:t>
   </x:si>
   <x:si>
     <x:t>2.13</x:t>
   </x:si>
   <x:si>
-    <x:t>BYBJ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem Finisar Dual Rate 10G/25G SR SFP28 Transceiver</x:t>
+    <x:t>C1YH</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem SR630 V4 x16/x16 PCIe Gen5 Cable Riser 1</x:t>
   </x:si>
   <x:si>
     <x:t>2.14</x:t>
   </x:si>
   <x:si>
-    <x:t>C1YH</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem SR630 V4 x16/x16 PCIe Gen5 Cable Riser 1</x:t>
+    <x:t>C1Z7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem SR630 V4 Full Height+Low Profile Riser1 Cage</x:t>
   </x:si>
   <x:si>
     <x:t>2.15</x:t>
   </x:si>
   <x:si>
-    <x:t>C1Z7</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem SR630 V4 Full Height+Low Profile Riser1 Cage</x:t>
+    <x:t>C0U8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 800W 230V/115V Platinum CRPS Hot-Swap Power Supply v1.5</x:t>
   </x:si>
   <x:si>
     <x:t>2.16</x:t>
   </x:si>
   <x:si>
-    <x:t>C0U8</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 800W 230V/115V Platinum CRPS Hot-Swap Power Supply v1.5</x:t>
+    <x:t>6400</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2.8m, 13A/100-250V, C13 to C14 Jumper Cord</x:t>
   </x:si>
   <x:si>
     <x:t>2.17</x:t>
   </x:si>
   <x:si>
-    <x:t>6400</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2.8m, 13A/100-250V, C13 to C14 Jumper Cord</x:t>
+    <x:t>C1YT</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 1U V4 Performance Fan Module</x:t>
   </x:si>
   <x:si>
     <x:t>2.18</x:t>
   </x:si>
   <x:si>
-    <x:t>C1YT</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 1U V4 Performance Fan Module</x:t>
+    <x:t>C1YP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 1U V4 Standard Media Bay</x:t>
   </x:si>
   <x:si>
     <x:t>2.19</x:t>
   </x:si>
   <x:si>
-    <x:t>C1YP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 1U V4 Standard Media Bay</x:t>
+    <x:t>C2DL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem Toolless Slide Rail Kit V4 with 1U CMA</x:t>
   </x:si>
   <x:si>
     <x:t>2.20</x:t>
   </x:si>
   <x:si>
-    <x:t>C2DL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem Toolless Slide Rail Kit V4 with 1U CMA</x:t>
+    <x:t>BPKR</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TPM 2.0</x:t>
   </x:si>
   <x:si>
     <x:t>2.21</x:t>
   </x:si>
   <x:si>
-    <x:t>BPKR</x:t>
-  </x:si>
-  <x:si>
-    <x:t>TPM 2.0</x:t>
+    <x:t>B7XZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Disable IPMI-over-LAN</x:t>
   </x:si>
   <x:si>
     <x:t>2.22</x:t>
   </x:si>
   <x:si>
-    <x:t>B7XZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Disable IPMI-over-LAN</x:t>
+    <x:t>BK15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>High voltage (200V+)</x:t>
   </x:si>
   <x:si>
     <x:t>2.23</x:t>
   </x:si>
   <x:si>
-    <x:t>BK15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>High voltage (200V+)</x:t>
+    <x:t>BZ7F</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem WW Lenovo LPK, Birch Stream</x:t>
   </x:si>
   <x:si>
     <x:t>2.24</x:t>
   </x:si>
   <x:si>
-    <x:t>BZ7F</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem WW Lenovo LPK, Birch Stream</x:t>
+    <x:t>B97B</x:t>
+  </x:si>
+  <x:si>
+    <x:t>XCC Label</x:t>
   </x:si>
   <x:si>
     <x:t>2.25</x:t>
   </x:si>
   <x:si>
-    <x:t>B97B</x:t>
-  </x:si>
-  <x:si>
-    <x:t>XCC Label</x:t>
+    <x:t>C212</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem BHS SR630 V4 1U PCIe number 1-2 and OCP number Label (BF+Rear M.2)</x:t>
   </x:si>
   <x:si>
     <x:t>2.26</x:t>
   </x:si>
   <x:si>
-    <x:t>C212</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem BHS SR630 V4 1U PCIe number 1-2 and OCP number Label (BF+Rear M.2)</x:t>
+    <x:t>C20N</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 800W rating label WW (CRPS) power</x:t>
   </x:si>
   <x:si>
     <x:t>2.27</x:t>
   </x:si>
   <x:si>
-    <x:t>C20N</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 800W rating label WW (CRPS) power</x:t>
+    <x:t>AWF9</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem Response time Service Label LI</x:t>
   </x:si>
   <x:si>
     <x:t>2.28</x:t>
   </x:si>
   <x:si>
-    <x:t>AWF9</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem Response time Service Label LI</x:t>
+    <x:t>C20D</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem SR630 V4 model Label name</x:t>
   </x:si>
   <x:si>
     <x:t>2.29</x:t>
   </x:si>
   <x:si>
-    <x:t>C20D</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem SR630 V4 model Label name</x:t>
+    <x:t>C20J</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem SR630 V4 Service Label for WW</x:t>
   </x:si>
   <x:si>
     <x:t>2.30</x:t>
   </x:si>
   <x:si>
-    <x:t>C20J</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem SR630 V4 Service Label for WW</x:t>
+    <x:t>AUTQ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem small Lenovo Label for 24x2.5"/12x3.5"/10x2.5"</x:t>
   </x:si>
   <x:si>
     <x:t>2.31</x:t>
   </x:si>
   <x:si>
-    <x:t>AUTQ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem small Lenovo Label for 24x2.5"/12x3.5"/10x2.5"</x:t>
+    <x:t>BQPS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem logo Label</x:t>
   </x:si>
   <x:si>
     <x:t>2.32</x:t>
   </x:si>
   <x:si>
-    <x:t>BQPS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem logo Label</x:t>
+    <x:t>C20B</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem SR630 V4 Agency label with CCC&amp;CECP</x:t>
   </x:si>
   <x:si>
     <x:t>2.33</x:t>
   </x:si>
   <x:si>
-    <x:t>C20B</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem SR630 V4 Agency label with CCC&amp;CECP</x:t>
+    <x:t>C21A</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem M.2 Power Cable, 2x10P 1.0PH-2x10P 1.25PH, 320mm</x:t>
   </x:si>
   <x:si>
     <x:t>2.34</x:t>
   </x:si>
   <x:si>
-    <x:t>C21A</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem M.2 Power Cable, 2x10P 1.0PH-2x10P 1.25PH, 320mm</x:t>
+    <x:t>C1Y4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem M.2 singal Cable, SLX4-MCIOX4, 310mm</x:t>
   </x:si>
   <x:si>
     <x:t>2.35</x:t>
   </x:si>
   <x:si>
-    <x:t>C1Y4</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem M.2 singal Cable, SLX4-MCIOX4, 310mm</x:t>
+    <x:t>BE0F</x:t>
+  </x:si>
+  <x:si>
+    <x:t>N+N Redundancy Without Over-Subscription</x:t>
   </x:si>
   <x:si>
     <x:t>2.36</x:t>
   </x:si>
   <x:si>
-    <x:t>BE0F</x:t>
-  </x:si>
-  <x:si>
-    <x:t>N+N Redundancy Without Over-Subscription</x:t>
+    <x:t>CAR5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SR630 V4 Laser service indicator</x:t>
   </x:si>
   <x:si>
     <x:t>2.37</x:t>
   </x:si>
   <x:si>
-    <x:t>CAR5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SR630 V4 Laser service indicator</x:t>
+    <x:t>C3NP</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem SR630 V4 MI-BF Cbl Riser to P9</x:t>
   </x:si>
   <x:si>
     <x:t>2.38</x:t>
   </x:si>
   <x:si>
-    <x:t>C3NP</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem SR630 V4 MI-BF Cbl Riser to P9</x:t>
+    <x:t>B0ML</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Feature Enable TPM MB on</x:t>
   </x:si>
   <x:si>
     <x:t>2.39</x:t>
   </x:si>
   <x:si>
-    <x:t>B0ML</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Feature Enable TPM MB on</x:t>
+    <x:t>C4DV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem SR630 V4 Processor Board</x:t>
   </x:si>
   <x:si>
     <x:t>2.40</x:t>
   </x:si>
   <x:si>
-    <x:t>C4DV</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem SR630 V4 Processor Board</x:t>
+    <x:t>C3K9</x:t>
+  </x:si>
+  <x:si>
+    <x:t>XClarity Platinum Upgrade v3</x:t>
   </x:si>
   <x:si>
     <x:t>2.41</x:t>
   </x:si>
   <x:si>
-    <x:t>C3K9</x:t>
-  </x:si>
-  <x:si>
-    <x:t>XClarity Platinum Upgrade v3</x:t>
+    <x:t>BEYJ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem MS Height CPU Dummy</x:t>
   </x:si>
   <x:si>
     <x:t>2.42</x:t>
   </x:si>
   <x:si>
-    <x:t>BEYJ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem MS Height CPU Dummy</x:t>
+    <x:t>AURS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lenovo ThinkSystem Memory Dummy</x:t>
   </x:si>
   <x:si>
     <x:t>2.43</x:t>
   </x:si>
   <x:si>
-    <x:t>AURS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lenovo ThinkSystem Memory Dummy</x:t>
+    <x:t>BCEB</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 1U V2 2x3 2.5" HDD Dummy</x:t>
   </x:si>
   <x:si>
     <x:t>2.44</x:t>
   </x:si>
   <x:si>
-    <x:t>BCEB</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 1U V2 2x3 2.5" HDD Dummy</x:t>
+    <x:t>AVEN</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 1x1 2.5" HDD Filler</x:t>
   </x:si>
   <x:si>
     <x:t>2.45</x:t>
   </x:si>
   <x:si>
-    <x:t>AVEN</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 1x1 2.5" HDD Filler</x:t>
+    <x:t>BPP5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>OCP3.0 Filler with screw</x:t>
   </x:si>
   <x:si>
     <x:t>2.46</x:t>
   </x:si>
   <x:si>
-    <x:t>BPP5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>OCP3.0 Filler with screw</x:t>
+    <x:t>B8NK</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 1U Super Cap Holder Dummy</x:t>
   </x:si>
   <x:si>
     <x:t>2.47</x:t>
   </x:si>
   <x:si>
-    <x:t>B8NK</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 1U Super Cap Holder Dummy</x:t>
+    <x:t>C1YZ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 1U V4 Fan filler</x:t>
   </x:si>
   <x:si>
     <x:t>2.48</x:t>
   </x:si>
   <x:si>
-    <x:t>C1YZ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 1U V4 Fan filler</x:t>
+    <x:t>BU1E</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Top Choice flag</x:t>
   </x:si>
   <x:si>
     <x:t>2.49</x:t>
   </x:si>
   <x:si>
-    <x:t>BU1E</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Top Choice flag</x:t>
+    <x:t>CA7N</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem SR630 V4 System I/O board v2</x:t>
   </x:si>
   <x:si>
     <x:t>2.50</x:t>
   </x:si>
   <x:si>
-    <x:t>CA7N</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem SR630 V4 System I/O board v2</x:t>
+    <x:t>C26Y</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem V4 CPU HS Clip</x:t>
   </x:si>
   <x:si>
     <x:t>2.51</x:t>
   </x:si>
   <x:si>
-    <x:t>C26Y</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem V4 CPU HS Clip</x:t>
+    <x:t>C1YV</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 1U V4 Rear Hot Swap M.2 Cage</x:t>
   </x:si>
   <x:si>
     <x:t>2.52</x:t>
   </x:si>
   <x:si>
-    <x:t>C1YV</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 1U V4 Rear Hot Swap M.2 Cage</x:t>
+    <x:t>C1LL</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem Rear M.2 HS Tray</x:t>
   </x:si>
   <x:si>
     <x:t>2.53</x:t>
   </x:si>
   <x:si>
-    <x:t>C1LL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem Rear M.2 HS Tray</x:t>
+    <x:t>CCWX</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hot-Swap M.2 Drive Interposer</x:t>
   </x:si>
   <x:si>
     <x:t>2.54</x:t>
   </x:si>
   <x:si>
-    <x:t>CCWX</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hot-Swap M.2 Drive Interposer</x:t>
+    <x:t>C2RD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem Hot Swap M.2 2280 SSD HeatSink</x:t>
   </x:si>
   <x:si>
     <x:t>2.55</x:t>
   </x:si>
   <x:si>
-    <x:t>C2RD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem Hot Swap M.2 2280 SSD HeatSink</x:t>
+    <x:t>C5XG</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem SR630 V4 General Config PKG AC+CL</x:t>
   </x:si>
   <x:si>
     <x:t>2.56</x:t>
   </x:si>
   <x:si>
-    <x:t>C5XG</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem SR630 V4 General Config PKG AC+CL</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2.57</x:t>
-  </x:si>
-  <x:si>
     <x:t>BTTY</x:t>
   </x:si>
   <x:si>
@@ -639,18 +636,15 @@
     <x:t>3.01</x:t>
   </x:si>
   <x:si>
+    <x:t>3444</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Registration only</x:t>
+  </x:si>
+  <x:si>
     <x:t>3.02</x:t>
   </x:si>
   <x:si>
-    <x:t>3444</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Registration only</x:t>
-  </x:si>
-  <x:si>
-    <x:t>3.03</x:t>
-  </x:si>
-  <x:si>
     <x:t>1340</x:t>
   </x:si>
   <x:si>
@@ -669,9 +663,6 @@
     <x:t>4.01</x:t>
   </x:si>
   <x:si>
-    <x:t>4.02</x:t>
-  </x:si>
-  <x:si>
     <x:t>SCY0</x:t>
   </x:si>
   <x:si>
@@ -690,36 +681,33 @@
     <x:t>5.01</x:t>
   </x:si>
   <x:si>
+    <x:t>QAJQ</x:t>
+  </x:si>
+  <x:si>
+    <x:t>SR630 V4</x:t>
+  </x:si>
+  <x:si>
     <x:t>5.02</x:t>
   </x:si>
   <x:si>
-    <x:t>QAJQ</x:t>
-  </x:si>
-  <x:si>
-    <x:t>SR630 V4</x:t>
+    <x:t>QA18</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Premier</x:t>
   </x:si>
   <x:si>
     <x:t>5.03</x:t>
   </x:si>
   <x:si>
-    <x:t>QA18</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Premier</x:t>
+    <x:t>QA0Y</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Months</x:t>
   </x:si>
   <x:si>
     <x:t>5.04</x:t>
   </x:si>
   <x:si>
-    <x:t>QA0Y</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Months</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.05</x:t>
-  </x:si>
-  <x:si>
     <x:t>QA11</x:t>
   </x:si>
   <x:si>
@@ -741,9 +729,6 @@
     <x:t>6.02</x:t>
   </x:si>
   <x:si>
-    <x:t>6.03</x:t>
-  </x:si>
-  <x:si>
     <x:t>QA1T</x:t>
   </x:si>
   <x:si>
@@ -765,18 +750,15 @@
     <x:t>7.02</x:t>
   </x:si>
   <x:si>
+    <x:t>QAK6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KYD</x:t>
+  </x:si>
+  <x:si>
     <x:t>7.03</x:t>
   </x:si>
   <x:si>
-    <x:t>QAK6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KYD</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7.04</x:t>
-  </x:si>
-  <x:si>
     <x:t>8</x:t>
   </x:si>
   <x:si>
@@ -801,27 +783,27 @@
     <x:t>9.04</x:t>
   </x:si>
   <x:si>
+    <x:t>C5R6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Intel Xeon 6507P 8C 150W 3.5GHz Processor</x:t>
+  </x:si>
+  <x:si>
     <x:t>9.05</x:t>
   </x:si>
   <x:si>
-    <x:t>C5R6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Intel Xeon 6507P 8C 150W 3.5GHz Processor</x:t>
-  </x:si>
-  <x:si>
     <x:t>9.06</x:t>
   </x:si>
   <x:si>
+    <x:t>C0U2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem 16GB TruDDR5 6400MHz (1Rx8) RDIMM</x:t>
+  </x:si>
+  <x:si>
     <x:t>9.07</x:t>
   </x:si>
   <x:si>
-    <x:t>C0U2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem 16GB TruDDR5 6400MHz (1Rx8) RDIMM</x:t>
-  </x:si>
-  <x:si>
     <x:t>9.08</x:t>
   </x:si>
   <x:si>
@@ -831,15 +813,15 @@
     <x:t>9.10</x:t>
   </x:si>
   <x:si>
+    <x:t>C4HU</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ThinkSystem Intel E610-T4 10GBase-T 4-Port OCP Ethernet Adapter(Generic FW)</x:t>
+  </x:si>
+  <x:si>
     <x:t>9.11</x:t>
   </x:si>
   <x:si>
-    <x:t>C4HU</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ThinkSystem Intel E610-T4 10GBase-T 4-Port OCP Ethernet Adapter(Generic FW)</x:t>
-  </x:si>
-  <x:si>
     <x:t>9.12</x:t>
   </x:si>
   <x:si>
@@ -969,21 +951,18 @@
     <x:t>9.54</x:t>
   </x:si>
   <x:si>
+    <x:t>BHSS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MI for PXE with RJ45 Network port</x:t>
+  </x:si>
+  <x:si>
     <x:t>9.55</x:t>
   </x:si>
   <x:si>
-    <x:t>BHSS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MI for PXE with RJ45 Network port</x:t>
-  </x:si>
-  <x:si>
     <x:t>9.56</x:t>
   </x:si>
   <x:si>
-    <x:t>9.57</x:t>
-  </x:si>
-  <x:si>
     <x:t>10</x:t>
   </x:si>
   <x:si>
@@ -993,9 +972,6 @@
     <x:t>10.02</x:t>
   </x:si>
   <x:si>
-    <x:t>10.03</x:t>
-  </x:si>
-  <x:si>
     <x:t>11</x:t>
   </x:si>
   <x:si>
@@ -1008,12 +984,6 @@
     <x:t>11.01</x:t>
   </x:si>
   <x:si>
-    <x:t>Veeam Data Platform FNDN Veeam Data Platform Foundation Universal Subscription License. Includes Enterprise Plus</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11.02</x:t>
-  </x:si>
-  <x:si>
     <x:t>SBRS</x:t>
   </x:si>
   <x:si>
@@ -1026,9 +996,6 @@
     <x:t>12.01</x:t>
   </x:si>
   <x:si>
-    <x:t>12.02</x:t>
-  </x:si>
-  <x:si>
     <x:t>13</x:t>
   </x:si>
   <x:si>
@@ -1044,9 +1011,6 @@
     <x:t>13.04</x:t>
   </x:si>
   <x:si>
-    <x:t>13.05</x:t>
-  </x:si>
-  <x:si>
     <x:t>14</x:t>
   </x:si>
   <x:si>
@@ -1056,9 +1020,6 @@
     <x:t>14.02</x:t>
   </x:si>
   <x:si>
-    <x:t>14.03</x:t>
-  </x:si>
-  <x:si>
     <x:t>15</x:t>
   </x:si>
   <x:si>
@@ -1069,9 +1030,6 @@
   </x:si>
   <x:si>
     <x:t>15.03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>15.04</x:t>
   </x:si>
   <x:si>
     <x:t>*</x:t>
@@ -1432,7 +1390,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:AA168"/>
+  <x:dimension ref="A1:AA155"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:27">
@@ -1571,13 +1529,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="0">
         <x:v>1E-06</x:v>
@@ -1585,16 +1543,16 @@
     </x:row>
     <x:row r="6" spans="1:27">
       <x:c r="A6" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F6" s="0">
         <x:v>1</x:v>
@@ -1605,16 +1563,16 @@
     </x:row>
     <x:row r="7" spans="1:27">
       <x:c r="A7" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F7" s="0">
         <x:v>1</x:v>
@@ -1625,16 +1583,16 @@
     </x:row>
     <x:row r="8" spans="1:27">
       <x:c r="A8" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="F8" s="0">
         <x:v>1</x:v>
@@ -1645,16 +1603,16 @@
     </x:row>
     <x:row r="9" spans="1:27">
       <x:c r="A9" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="F9" s="0">
         <x:v>1</x:v>
@@ -1665,19 +1623,19 @@
     </x:row>
     <x:row r="10" spans="1:27">
       <x:c r="A10" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="I10" s="0">
         <x:v>1E-06</x:v>
@@ -1685,19 +1643,19 @@
     </x:row>
     <x:row r="11" spans="1:27">
       <x:c r="A11" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I11" s="0">
         <x:v>1E-06</x:v>
@@ -1705,16 +1663,16 @@
     </x:row>
     <x:row r="12" spans="1:27">
       <x:c r="A12" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F12" s="0">
         <x:v>1</x:v>
@@ -1725,19 +1683,19 @@
     </x:row>
     <x:row r="13" spans="1:27">
       <x:c r="A13" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I13" s="0">
         <x:v>1E-06</x:v>
@@ -1745,19 +1703,19 @@
     </x:row>
     <x:row r="14" spans="1:27">
       <x:c r="A14" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="E14" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I14" s="0">
         <x:v>1E-06</x:v>
@@ -1765,16 +1723,16 @@
     </x:row>
     <x:row r="15" spans="1:27">
       <x:c r="A15" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E15" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F15" s="0">
         <x:v>1</x:v>
@@ -1785,19 +1743,19 @@
     </x:row>
     <x:row r="16" spans="1:27">
       <x:c r="A16" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E16" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I16" s="0">
         <x:v>1E-06</x:v>
@@ -1805,19 +1763,19 @@
     </x:row>
     <x:row r="17" spans="1:27">
       <x:c r="A17" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D17" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E17" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I17" s="0">
         <x:v>1E-06</x:v>
@@ -1825,16 +1783,16 @@
     </x:row>
     <x:row r="18" spans="1:27">
       <x:c r="A18" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D18" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="E18" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="F18" s="0">
         <x:v>1</x:v>
@@ -1845,19 +1803,19 @@
     </x:row>
     <x:row r="19" spans="1:27">
       <x:c r="A19" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D19" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I19" s="0">
         <x:v>1E-06</x:v>
@@ -1865,16 +1823,16 @@
     </x:row>
     <x:row r="20" spans="1:27">
       <x:c r="A20" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D20" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E20" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="F20" s="0">
         <x:v>2</x:v>
@@ -1885,19 +1843,19 @@
     </x:row>
     <x:row r="21" spans="1:27">
       <x:c r="A21" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D21" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="E21" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I21" s="0">
         <x:v>1E-06</x:v>
@@ -1905,19 +1863,19 @@
     </x:row>
     <x:row r="22" spans="1:27">
       <x:c r="A22" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D22" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="E22" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I22" s="0">
         <x:v>1E-06</x:v>
@@ -1925,16 +1883,16 @@
     </x:row>
     <x:row r="23" spans="1:27">
       <x:c r="A23" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D23" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="E23" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="F23" s="0">
         <x:v>1</x:v>
@@ -1945,16 +1903,16 @@
     </x:row>
     <x:row r="24" spans="1:27">
       <x:c r="A24" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D24" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E24" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="F24" s="0">
         <x:v>1</x:v>
@@ -1965,16 +1923,16 @@
     </x:row>
     <x:row r="25" spans="1:27">
       <x:c r="A25" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D25" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="E25" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="F25" s="0">
         <x:v>1</x:v>
@@ -1985,16 +1943,16 @@
     </x:row>
     <x:row r="26" spans="1:27">
       <x:c r="A26" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D26" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="E26" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="F26" s="0">
         <x:v>1</x:v>
@@ -2005,16 +1963,16 @@
     </x:row>
     <x:row r="27" spans="1:27">
       <x:c r="A27" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B27" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D27" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="E27" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="F27" s="0">
         <x:v>1</x:v>
@@ -2025,16 +1983,16 @@
     </x:row>
     <x:row r="28" spans="1:27">
       <x:c r="A28" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B28" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D28" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="E28" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="F28" s="0">
         <x:v>1</x:v>
@@ -2045,16 +2003,16 @@
     </x:row>
     <x:row r="29" spans="1:27">
       <x:c r="A29" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B29" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D29" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E29" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F29" s="0">
         <x:v>1</x:v>
@@ -2065,16 +2023,16 @@
     </x:row>
     <x:row r="30" spans="1:27">
       <x:c r="A30" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B30" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D30" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E30" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="F30" s="0">
         <x:v>1</x:v>
@@ -2085,16 +2043,16 @@
     </x:row>
     <x:row r="31" spans="1:27">
       <x:c r="A31" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B31" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D31" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E31" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="F31" s="0">
         <x:v>1</x:v>
@@ -2105,16 +2063,16 @@
     </x:row>
     <x:row r="32" spans="1:27">
       <x:c r="A32" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="B32" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D32" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="E32" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F32" s="0">
         <x:v>1</x:v>
@@ -2125,16 +2083,16 @@
     </x:row>
     <x:row r="33" spans="1:27">
       <x:c r="A33" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="B33" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D33" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="E33" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="F33" s="0">
         <x:v>1</x:v>
@@ -2145,16 +2103,16 @@
     </x:row>
     <x:row r="34" spans="1:27">
       <x:c r="A34" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B34" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E34" s="0" t="s">
-        <x:v>121</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="F34" s="0">
         <x:v>1</x:v>
@@ -2165,16 +2123,16 @@
     </x:row>
     <x:row r="35" spans="1:27">
       <x:c r="A35" s="0" t="s">
-        <x:v>122</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B35" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D35" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="E35" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F35" s="0">
         <x:v>1</x:v>
@@ -2185,16 +2143,16 @@
     </x:row>
     <x:row r="36" spans="1:27">
       <x:c r="A36" s="0" t="s">
-        <x:v>125</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B36" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D36" s="0" t="s">
-        <x:v>126</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E36" s="0" t="s">
-        <x:v>127</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="F36" s="0">
         <x:v>1</x:v>
@@ -2205,16 +2163,16 @@
     </x:row>
     <x:row r="37" spans="1:27">
       <x:c r="A37" s="0" t="s">
-        <x:v>128</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="B37" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D37" s="0" t="s">
-        <x:v>129</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E37" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F37" s="0">
         <x:v>1</x:v>
@@ -2225,16 +2183,16 @@
     </x:row>
     <x:row r="38" spans="1:27">
       <x:c r="A38" s="0" t="s">
-        <x:v>131</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B38" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D38" s="0" t="s">
-        <x:v>132</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="E38" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="F38" s="0">
         <x:v>1</x:v>
@@ -2245,16 +2203,16 @@
     </x:row>
     <x:row r="39" spans="1:27">
       <x:c r="A39" s="0" t="s">
-        <x:v>134</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="B39" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D39" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="E39" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="F39" s="0">
         <x:v>1</x:v>
@@ -2265,16 +2223,16 @@
     </x:row>
     <x:row r="40" spans="1:27">
       <x:c r="A40" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B40" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D40" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="E40" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="F40" s="0">
         <x:v>1</x:v>
@@ -2285,16 +2243,16 @@
     </x:row>
     <x:row r="41" spans="1:27">
       <x:c r="A41" s="0" t="s">
-        <x:v>140</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="B41" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D41" s="0" t="s">
-        <x:v>141</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="E41" s="0" t="s">
-        <x:v>142</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="F41" s="0">
         <x:v>1</x:v>
@@ -2305,16 +2263,16 @@
     </x:row>
     <x:row r="42" spans="1:27">
       <x:c r="A42" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="B42" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D42" s="0" t="s">
-        <x:v>144</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="E42" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="F42" s="0">
         <x:v>1</x:v>
@@ -2325,16 +2283,16 @@
     </x:row>
     <x:row r="43" spans="1:27">
       <x:c r="A43" s="0" t="s">
-        <x:v>146</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B43" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D43" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E43" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="F43" s="0">
         <x:v>1</x:v>
@@ -2345,16 +2303,16 @@
     </x:row>
     <x:row r="44" spans="1:27">
       <x:c r="A44" s="0" t="s">
-        <x:v>149</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B44" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D44" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="E44" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="F44" s="0">
         <x:v>1</x:v>
@@ -2365,16 +2323,16 @@
     </x:row>
     <x:row r="45" spans="1:27">
       <x:c r="A45" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B45" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D45" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="E45" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="F45" s="0">
         <x:v>1</x:v>
@@ -2385,19 +2343,19 @@
     </x:row>
     <x:row r="46" spans="1:27">
       <x:c r="A46" s="0" t="s">
-        <x:v>155</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B46" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D46" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="E46" s="0" t="s">
-        <x:v>157</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="F46" s="0">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="I46" s="0">
         <x:v>1E-06</x:v>
@@ -2405,19 +2363,19 @@
     </x:row>
     <x:row r="47" spans="1:27">
       <x:c r="A47" s="0" t="s">
-        <x:v>158</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="B47" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D47" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="E47" s="0" t="s">
-        <x:v>160</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="F47" s="0">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I47" s="0">
         <x:v>1E-06</x:v>
@@ -2425,19 +2383,19 @@
     </x:row>
     <x:row r="48" spans="1:27">
       <x:c r="A48" s="0" t="s">
-        <x:v>161</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="B48" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D48" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="E48" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="F48" s="0">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I48" s="0">
         <x:v>1E-06</x:v>
@@ -2445,19 +2403,19 @@
     </x:row>
     <x:row r="49" spans="1:27">
       <x:c r="A49" s="0" t="s">
-        <x:v>164</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B49" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D49" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="E49" s="0" t="s">
-        <x:v>166</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="F49" s="0">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I49" s="0">
         <x:v>1E-06</x:v>
@@ -2465,16 +2423,16 @@
     </x:row>
     <x:row r="50" spans="1:27">
       <x:c r="A50" s="0" t="s">
-        <x:v>167</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B50" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D50" s="0" t="s">
-        <x:v>168</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="E50" s="0" t="s">
-        <x:v>169</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F50" s="0">
         <x:v>1</x:v>
@@ -2485,16 +2443,16 @@
     </x:row>
     <x:row r="51" spans="1:27">
       <x:c r="A51" s="0" t="s">
-        <x:v>170</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B51" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D51" s="0" t="s">
-        <x:v>171</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="E51" s="0" t="s">
-        <x:v>172</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="F51" s="0">
         <x:v>1</x:v>
@@ -2505,16 +2463,16 @@
     </x:row>
     <x:row r="52" spans="1:27">
       <x:c r="A52" s="0" t="s">
-        <x:v>173</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B52" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D52" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="E52" s="0" t="s">
-        <x:v>175</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="F52" s="0">
         <x:v>1</x:v>
@@ -2525,16 +2483,16 @@
     </x:row>
     <x:row r="53" spans="1:27">
       <x:c r="A53" s="0" t="s">
-        <x:v>176</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B53" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D53" s="0" t="s">
-        <x:v>177</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="E53" s="0" t="s">
-        <x:v>178</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="F53" s="0">
         <x:v>1</x:v>
@@ -2545,16 +2503,16 @@
     </x:row>
     <x:row r="54" spans="1:27">
       <x:c r="A54" s="0" t="s">
-        <x:v>179</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B54" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D54" s="0" t="s">
-        <x:v>180</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="E54" s="0" t="s">
-        <x:v>181</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="F54" s="0">
         <x:v>1</x:v>
@@ -2565,16 +2523,16 @@
     </x:row>
     <x:row r="55" spans="1:27">
       <x:c r="A55" s="0" t="s">
-        <x:v>182</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="B55" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D55" s="0" t="s">
-        <x:v>183</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="E55" s="0" t="s">
-        <x:v>184</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="F55" s="0">
         <x:v>1</x:v>
@@ -2585,19 +2543,19 @@
     </x:row>
     <x:row r="56" spans="1:27">
       <x:c r="A56" s="0" t="s">
-        <x:v>185</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="B56" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D56" s="0" t="s">
-        <x:v>186</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="E56" s="0" t="s">
-        <x:v>187</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="F56" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I56" s="0">
         <x:v>1E-06</x:v>
@@ -2605,16 +2563,16 @@
     </x:row>
     <x:row r="57" spans="1:27">
       <x:c r="A57" s="0" t="s">
-        <x:v>188</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="B57" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D57" s="0" t="s">
-        <x:v>189</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="E57" s="0" t="s">
-        <x:v>190</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="F57" s="0">
         <x:v>2</x:v>
@@ -2625,16 +2583,16 @@
     </x:row>
     <x:row r="58" spans="1:27">
       <x:c r="A58" s="0" t="s">
-        <x:v>191</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="B58" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D58" s="0" t="s">
-        <x:v>192</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="E58" s="0" t="s">
-        <x:v>193</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="F58" s="0">
         <x:v>2</x:v>
@@ -2645,19 +2603,19 @@
     </x:row>
     <x:row r="59" spans="1:27">
       <x:c r="A59" s="0" t="s">
-        <x:v>194</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="B59" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D59" s="0" t="s">
-        <x:v>195</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="E59" s="0" t="s">
-        <x:v>196</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="F59" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I59" s="0">
         <x:v>1E-06</x:v>
@@ -2665,16 +2623,16 @@
     </x:row>
     <x:row r="60" spans="1:27">
       <x:c r="A60" s="0" t="s">
-        <x:v>197</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="B60" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D60" s="0" t="s">
-        <x:v>198</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="E60" s="0" t="s">
-        <x:v>199</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="F60" s="0">
         <x:v>1</x:v>
@@ -2685,19 +2643,19 @@
     </x:row>
     <x:row r="61" spans="1:27">
       <x:c r="A61" s="0" t="s">
-        <x:v>200</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="B61" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D61" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="E61" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="F61" s="0">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="I61" s="0">
         <x:v>1E-06</x:v>
@@ -2705,19 +2663,19 @@
     </x:row>
     <x:row r="62" spans="1:27">
       <x:c r="A62" s="0" t="s">
-        <x:v>203</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="B62" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D62" s="0" t="s">
-        <x:v>204</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="E62" s="0" t="s">
-        <x:v>205</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="F62" s="0">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I62" s="0">
         <x:v>1E-06</x:v>
@@ -2725,19 +2683,19 @@
     </x:row>
     <x:row r="63" spans="1:27">
       <x:c r="A63" s="0" t="s">
-        <x:v>206</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="B63" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D63" s="0" t="s">
-        <x:v>204</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="E63" s="0" t="s">
-        <x:v>205</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="F63" s="0">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I63" s="0">
         <x:v>1E-06</x:v>
@@ -2745,19 +2703,19 @@
     </x:row>
     <x:row r="64" spans="1:27">
       <x:c r="A64" s="0" t="s">
-        <x:v>207</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="B64" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D64" s="0" t="s">
-        <x:v>208</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="E64" s="0" t="s">
-        <x:v>209</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="F64" s="0">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="I64" s="0">
         <x:v>1E-06</x:v>
@@ -2765,16 +2723,16 @@
     </x:row>
     <x:row r="65" spans="1:27">
       <x:c r="A65" s="0" t="s">
-        <x:v>210</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="B65" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D65" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="E65" s="0" t="s">
-        <x:v>212</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="F65" s="0">
         <x:v>1</x:v>
@@ -2785,16 +2743,16 @@
     </x:row>
     <x:row r="66" spans="1:27">
       <x:c r="A66" s="0" t="s">
-        <x:v>213</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="B66" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D66" s="0" t="s">
-        <x:v>214</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="E66" s="0" t="s">
-        <x:v>215</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="F66" s="0">
         <x:v>8</x:v>
@@ -2805,19 +2763,19 @@
     </x:row>
     <x:row r="67" spans="1:27">
       <x:c r="A67" s="0" t="s">
-        <x:v>216</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="B67" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D67" s="0" t="s">
-        <x:v>214</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="E67" s="0" t="s">
-        <x:v>215</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F67" s="0">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I67" s="0">
         <x:v>1E-06</x:v>
@@ -2825,16 +2783,16 @@
     </x:row>
     <x:row r="68" spans="1:27">
       <x:c r="A68" s="0" t="s">
-        <x:v>217</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="B68" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D68" s="0" t="s">
-        <x:v>218</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="E68" s="0" t="s">
-        <x:v>219</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="F68" s="0">
         <x:v>1</x:v>
@@ -2845,19 +2803,19 @@
     </x:row>
     <x:row r="69" spans="1:27">
       <x:c r="A69" s="0" t="s">
-        <x:v>220</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="B69" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D69" s="0" t="s">
-        <x:v>221</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="E69" s="0" t="s">
-        <x:v>222</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="F69" s="0">
-        <x:v>8</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="I69" s="0">
         <x:v>1E-06</x:v>
@@ -2865,19 +2823,19 @@
     </x:row>
     <x:row r="70" spans="1:27">
       <x:c r="A70" s="0" t="s">
-        <x:v>223</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="B70" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D70" s="0" t="s">
-        <x:v>221</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="E70" s="0" t="s">
-        <x:v>222</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="F70" s="0">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I70" s="0">
         <x:v>1E-06</x:v>
@@ -2885,19 +2843,19 @@
     </x:row>
     <x:row r="71" spans="1:27">
       <x:c r="A71" s="0" t="s">
-        <x:v>224</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="B71" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D71" s="0" t="s">
-        <x:v>225</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="E71" s="0" t="s">
-        <x:v>226</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="F71" s="0">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="I71" s="0">
         <x:v>1E-06</x:v>
@@ -2905,16 +2863,16 @@
     </x:row>
     <x:row r="72" spans="1:27">
       <x:c r="A72" s="0" t="s">
-        <x:v>227</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="B72" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D72" s="0" t="s">
-        <x:v>228</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="E72" s="0" t="s">
-        <x:v>229</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F72" s="0">
         <x:v>1</x:v>
@@ -2925,19 +2883,19 @@
     </x:row>
     <x:row r="73" spans="1:27">
       <x:c r="A73" s="0" t="s">
-        <x:v>230</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="B73" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D73" s="0" t="s">
-        <x:v>231</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="E73" s="0" t="s">
-        <x:v>232</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="F73" s="0">
-        <x:v>36</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I73" s="0">
         <x:v>1E-06</x:v>
@@ -2945,19 +2903,19 @@
     </x:row>
     <x:row r="74" spans="1:27">
       <x:c r="A74" s="0" t="s">
-        <x:v>233</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="B74" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D74" s="0" t="s">
-        <x:v>234</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="E74" s="0" t="s">
-        <x:v>235</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="F74" s="0">
-        <x:v>1</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="I74" s="0">
         <x:v>1E-06</x:v>
@@ -2965,19 +2923,19 @@
     </x:row>
     <x:row r="75" spans="1:27">
       <x:c r="A75" s="0" t="s">
-        <x:v>236</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="B75" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D75" s="0" t="s">
-        <x:v>237</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="E75" s="0" t="s">
-        <x:v>238</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F75" s="0">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I75" s="0">
         <x:v>1E-06</x:v>
@@ -2985,19 +2943,19 @@
     </x:row>
     <x:row r="76" spans="1:27">
       <x:c r="A76" s="0" t="s">
-        <x:v>239</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="B76" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D76" s="0" t="s">
-        <x:v>237</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="E76" s="0" t="s">
-        <x:v>238</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="F76" s="0">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I76" s="0">
         <x:v>1E-06</x:v>
@@ -3005,19 +2963,19 @@
     </x:row>
     <x:row r="77" spans="1:27">
       <x:c r="A77" s="0" t="s">
-        <x:v>240</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="B77" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D77" s="0" t="s">
-        <x:v>225</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="E77" s="0" t="s">
-        <x:v>226</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="F77" s="0">
-        <x:v>1</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="I77" s="0">
         <x:v>1E-06</x:v>
@@ -3025,39 +2983,39 @@
     </x:row>
     <x:row r="78" spans="1:27">
       <x:c r="A78" s="0" t="s">
-        <x:v>241</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="B78" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D78" s="0" t="s">
-        <x:v>242</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="E78" s="0" t="s">
-        <x:v>243</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="F78" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I78" s="0">
-        <x:v>1E-06</x:v>
+        <x:v>36348.82</x:v>
       </x:c>
     </x:row>
     <x:row r="79" spans="1:27">
       <x:c r="A79" s="0" t="s">
-        <x:v>244</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="B79" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D79" s="0" t="s">
-        <x:v>245</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E79" s="0" t="s">
-        <x:v>246</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="F79" s="0">
-        <x:v>8</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I79" s="0">
         <x:v>1E-06</x:v>
@@ -3065,19 +3023,19 @@
     </x:row>
     <x:row r="80" spans="1:27">
       <x:c r="A80" s="0" t="s">
-        <x:v>247</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="B80" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D80" s="0" t="s">
-        <x:v>245</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E80" s="0" t="s">
-        <x:v>246</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="F80" s="0">
-        <x:v>8</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I80" s="0">
         <x:v>1E-06</x:v>
@@ -3085,16 +3043,16 @@
     </x:row>
     <x:row r="81" spans="1:27">
       <x:c r="A81" s="0" t="s">
-        <x:v>248</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="B81" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D81" s="0" t="s">
-        <x:v>225</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E81" s="0" t="s">
-        <x:v>226</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F81" s="0">
         <x:v>1</x:v>
@@ -3105,16 +3063,16 @@
     </x:row>
     <x:row r="82" spans="1:27">
       <x:c r="A82" s="0" t="s">
-        <x:v>249</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="B82" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D82" s="0" t="s">
-        <x:v>250</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E82" s="0" t="s">
-        <x:v>251</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F82" s="0">
         <x:v>1</x:v>
@@ -3125,19 +3083,19 @@
     </x:row>
     <x:row r="83" spans="1:27">
       <x:c r="A83" s="0" t="s">
-        <x:v>252</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="B83" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D83" s="0" t="s">
-        <x:v>231</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="E83" s="0" t="s">
-        <x:v>232</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="F83" s="0">
-        <x:v>36</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I83" s="0">
         <x:v>1E-06</x:v>
@@ -3145,39 +3103,39 @@
     </x:row>
     <x:row r="84" spans="1:27">
       <x:c r="A84" s="0" t="s">
-        <x:v>253</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="B84" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D84" s="0" t="s">
-        <x:v>254</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="E84" s="0" t="s">
-        <x:v>254</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="F84" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I84" s="0">
-        <x:v>36348.82</x:v>
+        <x:v>1E-06</x:v>
       </x:c>
     </x:row>
     <x:row r="85" spans="1:27">
       <x:c r="A85" s="0" t="s">
-        <x:v>255</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="B85" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D85" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="E85" s="0" t="s">
-        <x:v>256</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="F85" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I85" s="0">
         <x:v>1E-06</x:v>
@@ -3185,19 +3143,19 @@
     </x:row>
     <x:row r="86" spans="1:27">
       <x:c r="A86" s="0" t="s">
-        <x:v>257</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="B86" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D86" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E86" s="0" t="s">
-        <x:v>256</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="F86" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I86" s="0">
         <x:v>1E-06</x:v>
@@ -3205,16 +3163,16 @@
     </x:row>
     <x:row r="87" spans="1:27">
       <x:c r="A87" s="0" t="s">
-        <x:v>258</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="B87" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D87" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E87" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F87" s="0">
         <x:v>1</x:v>
@@ -3225,19 +3183,19 @@
     </x:row>
     <x:row r="88" spans="1:27">
       <x:c r="A88" s="0" t="s">
-        <x:v>259</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="B88" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D88" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="E88" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="F88" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I88" s="0">
         <x:v>1E-06</x:v>
@@ -3245,16 +3203,16 @@
     </x:row>
     <x:row r="89" spans="1:27">
       <x:c r="A89" s="0" t="s">
-        <x:v>260</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="B89" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D89" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="E89" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="F89" s="0">
         <x:v>1</x:v>
@@ -3265,19 +3223,19 @@
     </x:row>
     <x:row r="90" spans="1:27">
       <x:c r="A90" s="0" t="s">
-        <x:v>261</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="B90" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D90" s="0" t="s">
-        <x:v>262</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E90" s="0" t="s">
-        <x:v>263</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F90" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I90" s="0">
         <x:v>1E-06</x:v>
@@ -3285,19 +3243,19 @@
     </x:row>
     <x:row r="91" spans="1:27">
       <x:c r="A91" s="0" t="s">
-        <x:v>264</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="B91" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D91" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E91" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F91" s="0">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I91" s="0">
         <x:v>1E-06</x:v>
@@ -3305,16 +3263,16 @@
     </x:row>
     <x:row r="92" spans="1:27">
       <x:c r="A92" s="0" t="s">
-        <x:v>265</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="B92" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D92" s="0" t="s">
-        <x:v>266</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E92" s="0" t="s">
-        <x:v>267</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="F92" s="0">
         <x:v>1</x:v>
@@ -3325,16 +3283,16 @@
     </x:row>
     <x:row r="93" spans="1:27">
       <x:c r="A93" s="0" t="s">
-        <x:v>268</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="B93" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D93" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="E93" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="F93" s="0">
         <x:v>1</x:v>
@@ -3345,19 +3303,19 @@
     </x:row>
     <x:row r="94" spans="1:27">
       <x:c r="A94" s="0" t="s">
-        <x:v>269</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="B94" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D94" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E94" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="F94" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I94" s="0">
         <x:v>1E-06</x:v>
@@ -3365,16 +3323,16 @@
     </x:row>
     <x:row r="95" spans="1:27">
       <x:c r="A95" s="0" t="s">
-        <x:v>270</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="B95" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D95" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E95" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="F95" s="0">
         <x:v>2</x:v>
@@ -3385,19 +3343,19 @@
     </x:row>
     <x:row r="96" spans="1:27">
       <x:c r="A96" s="0" t="s">
-        <x:v>271</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="B96" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D96" s="0" t="s">
-        <x:v>272</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="E96" s="0" t="s">
-        <x:v>273</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="F96" s="0">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I96" s="0">
         <x:v>1E-06</x:v>
@@ -3411,13 +3369,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D97" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="E97" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="F97" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I97" s="0">
         <x:v>1E-06</x:v>
@@ -3431,13 +3389,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D98" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="E98" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="F98" s="0">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I98" s="0">
         <x:v>1E-06</x:v>
@@ -3451,10 +3409,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D99" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="E99" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="F99" s="0">
         <x:v>1</x:v>
@@ -3471,10 +3429,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D100" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="E100" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="F100" s="0">
         <x:v>1</x:v>
@@ -3491,13 +3449,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D101" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="E101" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="F101" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I101" s="0">
         <x:v>1E-06</x:v>
@@ -3511,13 +3469,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D102" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="E102" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="F102" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I102" s="0">
         <x:v>1E-06</x:v>
@@ -3531,13 +3489,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D103" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="E103" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="F103" s="0">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I103" s="0">
         <x:v>1E-06</x:v>
@@ -3551,10 +3509,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D104" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E104" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F104" s="0">
         <x:v>1</x:v>
@@ -3571,10 +3529,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D105" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E105" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="F105" s="0">
         <x:v>1</x:v>
@@ -3591,10 +3549,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D106" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="E106" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="F106" s="0">
         <x:v>1</x:v>
@@ -3611,10 +3569,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D107" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="E107" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="F107" s="0">
         <x:v>1</x:v>
@@ -3631,10 +3589,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D108" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="E108" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="F108" s="0">
         <x:v>1</x:v>
@@ -3651,10 +3609,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D109" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="E109" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="F109" s="0">
         <x:v>1</x:v>
@@ -3671,10 +3629,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D110" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="E110" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="F110" s="0">
         <x:v>1</x:v>
@@ -3691,10 +3649,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D111" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="E111" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="F111" s="0">
         <x:v>1</x:v>
@@ -3711,10 +3669,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D112" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="E112" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="F112" s="0">
         <x:v>1</x:v>
@@ -3731,10 +3689,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D113" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="E113" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="F113" s="0">
         <x:v>1</x:v>
@@ -3751,10 +3709,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D114" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="E114" s="0" t="s">
-        <x:v>118</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="F114" s="0">
         <x:v>1</x:v>
@@ -3771,10 +3729,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D115" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="E115" s="0" t="s">
-        <x:v>121</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="F115" s="0">
         <x:v>1</x:v>
@@ -3791,10 +3749,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D116" s="0" t="s">
-        <x:v>123</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="E116" s="0" t="s">
-        <x:v>124</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="F116" s="0">
         <x:v>1</x:v>
@@ -3811,10 +3769,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D117" s="0" t="s">
-        <x:v>126</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="E117" s="0" t="s">
-        <x:v>127</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="F117" s="0">
         <x:v>1</x:v>
@@ -3831,10 +3789,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D118" s="0" t="s">
-        <x:v>129</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E118" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="F118" s="0">
         <x:v>1</x:v>
@@ -3851,10 +3809,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D119" s="0" t="s">
-        <x:v>132</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="E119" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="F119" s="0">
         <x:v>1</x:v>
@@ -3871,10 +3829,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D120" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="E120" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="F120" s="0">
         <x:v>1</x:v>
@@ -3891,10 +3849,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D121" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="E121" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="F121" s="0">
         <x:v>1</x:v>
@@ -3911,13 +3869,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D122" s="0" t="s">
-        <x:v>141</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="E122" s="0" t="s">
-        <x:v>142</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="F122" s="0">
-        <x:v>1</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I122" s="0">
         <x:v>1E-06</x:v>
@@ -3931,10 +3889,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D123" s="0" t="s">
-        <x:v>144</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="E123" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="F123" s="0">
         <x:v>1</x:v>
@@ -3951,10 +3909,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D124" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="E124" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="F124" s="0">
         <x:v>1</x:v>
@@ -3971,10 +3929,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D125" s="0" t="s">
-        <x:v>150</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="E125" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="F125" s="0">
         <x:v>1</x:v>
@@ -3991,10 +3949,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D126" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="E126" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="F126" s="0">
         <x:v>1</x:v>
@@ -4011,10 +3969,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D127" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="E127" s="0" t="s">
-        <x:v>157</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="F127" s="0">
         <x:v>1</x:v>
@@ -4031,10 +3989,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D128" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="E128" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="F128" s="0">
         <x:v>1</x:v>
@@ -4051,13 +4009,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D129" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="E129" s="0" t="s">
-        <x:v>166</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="F129" s="0">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I129" s="0">
         <x:v>1E-06</x:v>
@@ -4071,13 +4029,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D130" s="0" t="s">
-        <x:v>168</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="E130" s="0" t="s">
-        <x:v>169</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="F130" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I130" s="0">
         <x:v>1E-06</x:v>
@@ -4091,13 +4049,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D131" s="0" t="s">
-        <x:v>171</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="E131" s="0" t="s">
-        <x:v>172</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="F131" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I131" s="0">
         <x:v>1E-06</x:v>
@@ -4111,13 +4069,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D132" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="E132" s="0" t="s">
-        <x:v>175</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="F132" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I132" s="0">
         <x:v>1E-06</x:v>
@@ -4131,10 +4089,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="D133" s="0" t="s">
-        <x:v>177</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="E133" s="0" t="s">
-        <x:v>178</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="F133" s="0">
         <x:v>1</x:v>
@@ -4145,16 +4103,16 @@
     </x:row>
     <x:row r="134" spans="1:27">
       <x:c r="A134" s="0" t="s">
-        <x:v>311</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="B134" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D134" s="0" t="s">
-        <x:v>180</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="E134" s="0" t="s">
-        <x:v>181</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="F134" s="0">
         <x:v>1</x:v>
@@ -4165,16 +4123,16 @@
     </x:row>
     <x:row r="135" spans="1:27">
       <x:c r="A135" s="0" t="s">
-        <x:v>312</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="B135" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D135" s="0" t="s">
-        <x:v>183</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="E135" s="0" t="s">
-        <x:v>184</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="F135" s="0">
         <x:v>1</x:v>
@@ -4185,19 +4143,19 @@
     </x:row>
     <x:row r="136" spans="1:27">
       <x:c r="A136" s="0" t="s">
-        <x:v>313</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="B136" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D136" s="0" t="s">
-        <x:v>186</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="E136" s="0" t="s">
-        <x:v>187</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="F136" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I136" s="0">
         <x:v>1E-06</x:v>
@@ -4205,19 +4163,19 @@
     </x:row>
     <x:row r="137" spans="1:27">
       <x:c r="A137" s="0" t="s">
-        <x:v>314</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="B137" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D137" s="0" t="s">
-        <x:v>189</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="E137" s="0" t="s">
-        <x:v>190</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="F137" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I137" s="0">
         <x:v>1E-06</x:v>
@@ -4225,19 +4183,19 @@
     </x:row>
     <x:row r="138" spans="1:27">
       <x:c r="A138" s="0" t="s">
-        <x:v>315</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="B138" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D138" s="0" t="s">
-        <x:v>192</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="E138" s="0" t="s">
-        <x:v>193</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="F138" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I138" s="0">
         <x:v>1E-06</x:v>
@@ -4245,16 +4203,16 @@
     </x:row>
     <x:row r="139" spans="1:27">
       <x:c r="A139" s="0" t="s">
-        <x:v>316</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="B139" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D139" s="0" t="s">
-        <x:v>195</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="E139" s="0" t="s">
-        <x:v>196</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="F139" s="0">
         <x:v>2</x:v>
@@ -4265,16 +4223,16 @@
     </x:row>
     <x:row r="140" spans="1:27">
       <x:c r="A140" s="0" t="s">
-        <x:v>317</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="B140" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D140" s="0" t="s">
-        <x:v>318</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="E140" s="0" t="s">
-        <x:v>319</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="F140" s="0">
         <x:v>1</x:v>
@@ -4285,19 +4243,19 @@
     </x:row>
     <x:row r="141" spans="1:27">
       <x:c r="A141" s="0" t="s">
-        <x:v>320</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="B141" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D141" s="0" t="s">
-        <x:v>198</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="E141" s="0" t="s">
-        <x:v>199</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="F141" s="0">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I141" s="0">
         <x:v>1E-06</x:v>
@@ -4305,16 +4263,16 @@
     </x:row>
     <x:row r="142" spans="1:27">
       <x:c r="A142" s="0" t="s">
-        <x:v>321</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="B142" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D142" s="0" t="s">
-        <x:v>201</x:v>
+        <x:v>215</x:v>
       </x:c>
       <x:c r="E142" s="0" t="s">
-        <x:v>202</x:v>
+        <x:v>216</x:v>
       </x:c>
       <x:c r="F142" s="0">
         <x:v>1</x:v>
@@ -4325,16 +4283,16 @@
     </x:row>
     <x:row r="143" spans="1:27">
       <x:c r="A143" s="0" t="s">
-        <x:v>322</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="B143" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D143" s="0" t="s">
-        <x:v>204</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="E143" s="0" t="s">
-        <x:v>205</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="F143" s="0">
         <x:v>2</x:v>
@@ -4345,19 +4303,19 @@
     </x:row>
     <x:row r="144" spans="1:27">
       <x:c r="A144" s="0" t="s">
-        <x:v>323</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="B144" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D144" s="0" t="s">
-        <x:v>204</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="E144" s="0" t="s">
-        <x:v>205</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F144" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I144" s="0">
         <x:v>1E-06</x:v>
@@ -4365,16 +4323,16 @@
     </x:row>
     <x:row r="145" spans="1:27">
       <x:c r="A145" s="0" t="s">
-        <x:v>324</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="B145" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D145" s="0" t="s">
-        <x:v>208</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="E145" s="0" t="s">
-        <x:v>209</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="F145" s="0">
         <x:v>1</x:v>
@@ -4385,19 +4343,19 @@
     </x:row>
     <x:row r="146" spans="1:27">
       <x:c r="A146" s="0" t="s">
-        <x:v>325</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="B146" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D146" s="0" t="s">
-        <x:v>211</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="E146" s="0" t="s">
-        <x:v>212</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="F146" s="0">
-        <x:v>1</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="I146" s="0">
         <x:v>1E-06</x:v>
@@ -4405,19 +4363,19 @@
     </x:row>
     <x:row r="147" spans="1:27">
       <x:c r="A147" s="0" t="s">
-        <x:v>326</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="B147" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D147" s="0" t="s">
-        <x:v>327</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="E147" s="0" t="s">
-        <x:v>328</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="F147" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I147" s="0">
         <x:v>1E-06</x:v>
@@ -4425,16 +4383,16 @@
     </x:row>
     <x:row r="148" spans="1:27">
       <x:c r="A148" s="0" t="s">
-        <x:v>329</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="B148" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D148" s="0" t="s">
-        <x:v>327</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="E148" s="0" t="s">
-        <x:v>330</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="F148" s="0">
         <x:v>2</x:v>
@@ -4445,16 +4403,16 @@
     </x:row>
     <x:row r="149" spans="1:27">
       <x:c r="A149" s="0" t="s">
-        <x:v>331</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="B149" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D149" s="0" t="s">
-        <x:v>332</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="E149" s="0" t="s">
-        <x:v>333</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F149" s="0">
         <x:v>1</x:v>
@@ -4465,19 +4423,19 @@
     </x:row>
     <x:row r="150" spans="1:27">
       <x:c r="A150" s="0" t="s">
-        <x:v>334</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="B150" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D150" s="0" t="s">
-        <x:v>214</x:v>
+        <x:v>237</x:v>
       </x:c>
       <x:c r="E150" s="0" t="s">
-        <x:v>215</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="F150" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I150" s="0">
         <x:v>1E-06</x:v>
@@ -4485,16 +4443,16 @@
     </x:row>
     <x:row r="151" spans="1:27">
       <x:c r="A151" s="0" t="s">
-        <x:v>335</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="B151" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D151" s="0" t="s">
-        <x:v>214</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="E151" s="0" t="s">
-        <x:v>215</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="F151" s="0">
         <x:v>2</x:v>
@@ -4505,16 +4463,16 @@
     </x:row>
     <x:row r="152" spans="1:27">
       <x:c r="A152" s="0" t="s">
-        <x:v>336</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="B152" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D152" s="0" t="s">
-        <x:v>218</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="E152" s="0" t="s">
-        <x:v>219</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="F152" s="0">
         <x:v>1</x:v>
@@ -4525,19 +4483,19 @@
     </x:row>
     <x:row r="153" spans="1:27">
       <x:c r="A153" s="0" t="s">
-        <x:v>337</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="B153" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
       <x:c r="D153" s="0" t="s">
-        <x:v>221</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="E153" s="0" t="s">
-        <x:v>222</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="F153" s="0">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I153" s="0">
         <x:v>1E-06</x:v>
@@ -4545,290 +4503,30 @@
     </x:row>
     <x:row r="154" spans="1:27">
       <x:c r="A154" s="0" t="s">
+        <x:v>337</x:v>
+      </x:c>
+      <x:c r="B154" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="D154" s="0" t="s">
+        <x:v>227</x:v>
+      </x:c>
+      <x:c r="E154" s="0" t="s">
+        <x:v>228</x:v>
+      </x:c>
+      <x:c r="F154" s="0">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="I154" s="0">
+        <x:v>1E-06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="155" spans="1:27">
+      <x:c r="B155" s="0" t="s">
         <x:v>338</x:v>
       </x:c>
-      <x:c r="B154" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D154" s="0" t="s">
-        <x:v>221</x:v>
-      </x:c>
-      <x:c r="E154" s="0" t="s">
-        <x:v>222</x:v>
-      </x:c>
-      <x:c r="F154" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="I154" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="155" spans="1:27">
-      <x:c r="A155" s="0" t="s">
+      <x:c r="D155" s="0" t="s">
         <x:v>339</x:v>
-      </x:c>
-      <x:c r="B155" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D155" s="0" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="E155" s="0" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="F155" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I155" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="156" spans="1:27">
-      <x:c r="A156" s="0" t="s">
-        <x:v>340</x:v>
-      </x:c>
-      <x:c r="B156" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D156" s="0" t="s">
-        <x:v>228</x:v>
-      </x:c>
-      <x:c r="E156" s="0" t="s">
-        <x:v>229</x:v>
-      </x:c>
-      <x:c r="F156" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I156" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="157" spans="1:27">
-      <x:c r="A157" s="0" t="s">
-        <x:v>341</x:v>
-      </x:c>
-      <x:c r="B157" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D157" s="0" t="s">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="E157" s="0" t="s">
-        <x:v>232</x:v>
-      </x:c>
-      <x:c r="F157" s="0">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="I157" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="158" spans="1:27">
-      <x:c r="A158" s="0" t="s">
-        <x:v>342</x:v>
-      </x:c>
-      <x:c r="B158" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D158" s="0" t="s">
-        <x:v>234</x:v>
-      </x:c>
-      <x:c r="E158" s="0" t="s">
-        <x:v>235</x:v>
-      </x:c>
-      <x:c r="F158" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I158" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="159" spans="1:27">
-      <x:c r="A159" s="0" t="s">
-        <x:v>343</x:v>
-      </x:c>
-      <x:c r="B159" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D159" s="0" t="s">
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="E159" s="0" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="F159" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="I159" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="160" spans="1:27">
-      <x:c r="A160" s="0" t="s">
-        <x:v>344</x:v>
-      </x:c>
-      <x:c r="B160" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D160" s="0" t="s">
-        <x:v>237</x:v>
-      </x:c>
-      <x:c r="E160" s="0" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="F160" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="I160" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="161" spans="1:27">
-      <x:c r="A161" s="0" t="s">
-        <x:v>345</x:v>
-      </x:c>
-      <x:c r="B161" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D161" s="0" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="E161" s="0" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="F161" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I161" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="162" spans="1:27">
-      <x:c r="A162" s="0" t="s">
-        <x:v>346</x:v>
-      </x:c>
-      <x:c r="B162" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D162" s="0" t="s">
-        <x:v>242</x:v>
-      </x:c>
-      <x:c r="E162" s="0" t="s">
-        <x:v>243</x:v>
-      </x:c>
-      <x:c r="F162" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I162" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="163" spans="1:27">
-      <x:c r="A163" s="0" t="s">
-        <x:v>347</x:v>
-      </x:c>
-      <x:c r="B163" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D163" s="0" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="E163" s="0" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="F163" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="I163" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="164" spans="1:27">
-      <x:c r="A164" s="0" t="s">
-        <x:v>348</x:v>
-      </x:c>
-      <x:c r="B164" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D164" s="0" t="s">
-        <x:v>245</x:v>
-      </x:c>
-      <x:c r="E164" s="0" t="s">
-        <x:v>246</x:v>
-      </x:c>
-      <x:c r="F164" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="I164" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="165" spans="1:27">
-      <x:c r="A165" s="0" t="s">
-        <x:v>349</x:v>
-      </x:c>
-      <x:c r="B165" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D165" s="0" t="s">
-        <x:v>225</x:v>
-      </x:c>
-      <x:c r="E165" s="0" t="s">
-        <x:v>226</x:v>
-      </x:c>
-      <x:c r="F165" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I165" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="166" spans="1:27">
-      <x:c r="A166" s="0" t="s">
-        <x:v>350</x:v>
-      </x:c>
-      <x:c r="B166" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D166" s="0" t="s">
-        <x:v>250</x:v>
-      </x:c>
-      <x:c r="E166" s="0" t="s">
-        <x:v>251</x:v>
-      </x:c>
-      <x:c r="F166" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I166" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="167" spans="1:27">
-      <x:c r="A167" s="0" t="s">
-        <x:v>351</x:v>
-      </x:c>
-      <x:c r="B167" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D167" s="0" t="s">
-        <x:v>231</x:v>
-      </x:c>
-      <x:c r="E167" s="0" t="s">
-        <x:v>232</x:v>
-      </x:c>
-      <x:c r="F167" s="0">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="I167" s="0">
-        <x:v>1E-06</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="168" spans="1:27">
-      <x:c r="B168" s="0" t="s">
-        <x:v>352</x:v>
-      </x:c>
-      <x:c r="D168" s="0" t="s">
-        <x:v>353</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>